<commit_message>
docs: calculate real SUNAT taxes and add pricing support sheet in financial plan
</commit_message>
<xml_diff>
--- a/ENTREGABLE/10. Estructura de Costos y Flujo de Caja/SportMatch_Connect_Financial_Plan.xlsx
+++ b/ENTREGABLE/10. Estructura de Costos y Flujo de Caja/SportMatch_Connect_Financial_Plan.xlsx
@@ -5,7 +5,7 @@
   <sheets>
     <sheet name="Inversión Inicial" sheetId="1" r:id="rId1"/>
     <sheet name="Costos AWS-Supabase" sheetId="2" r:id="rId2"/>
-    <sheet name="Gastos Operativos" sheetId="3" r:id="rId3"/>
+    <sheet name="Sustento de Precios" sheetId="3" r:id="rId3"/>
     <sheet name="Flujo de Caja Proyectado" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
@@ -1042,229 +1042,110 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SportMatch Connect - Estructura de Gastos Operativos Mensuales (Año 1)</v>
+        <v>SportMatch Connect - Sustento de Precios y Tarifas de la Empresa</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Conceptos de Negocio, Adquisición, Loyalty e Impuestos</v>
+        <v>Justificación Comercial de Monetización (B2B Comisiones &amp; B2C Suscripción Premium)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Concepto de Gasto</v>
+        <v>Línea de Ingreso</v>
       </c>
       <c r="B4" t="str">
-        <v>Sub-concepto</v>
+        <v>Tarifa (S/.)</v>
       </c>
       <c r="C4" t="str">
-        <v>Detalle Comercial / Empresa</v>
+        <v>Base de Cobro</v>
       </c>
       <c r="D4" t="str">
-        <v>Costo Mensual Propedéutico (S/.)</v>
+        <v>Justificación del Precio</v>
       </c>
       <c r="E4" t="str">
-        <v>Frecuencia</v>
+        <v>Beneficio Generado para el Cliente</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Infraestructura Nube</v>
+        <v>Comisión B2B (Complejos)</v>
       </c>
       <c r="B5" t="str">
-        <v>AWS &amp; Supabase</v>
+        <v>5.00%</v>
       </c>
       <c r="C5" t="str">
-        <v>Host de servidores NestJS, Postgres/PostGIS y CDN</v>
-      </c>
-      <c r="D5">
-        <v>893</v>
+        <v>Sobre el valor total de cada reserva</v>
+      </c>
+      <c r="D5" t="str">
+        <v>El precio promedio de alquiler de canchas en Lima Moderna es de S/. 90.00 por hora. Una comisión del 5% equivale a S/. 4.50. Este costo es absorbido por el recinto a cambio de incrementar su tasa de ocupación (de 35% a 65%) reduciendo sus horas muertas de lunes a viernes.</v>
       </c>
       <c r="E5" t="str">
-        <v>Mensual</v>
+        <v>Exposición de sus canchas libres ante miles de jugadores recreativos, panel administrativo de gestión de horarios gratuito y liquidación automatizada de fondos.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Marketing &amp; Adquisición</v>
+        <v>Suscripción B2C Premium</v>
       </c>
       <c r="B6" t="str">
-        <v>Meta Ads (FB/IG)</v>
+        <v>19.90</v>
       </c>
       <c r="C6" t="str">
-        <v>Campañas geolocalizadas dirigidas a deportistas recreativos en Lima</v>
-      </c>
-      <c r="D6">
-        <v>120</v>
+        <v>Mensual por usuario premium</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Equivale al costo de media cajetilla de cigarrillos o un café Starbucks, lo cual es sumamente asequible para deportistas recreativos concurrentes de NSE A, B y C en Lima.</v>
       </c>
       <c r="E6" t="str">
-        <v>Mensual</v>
+        <v>Acceso a reserva anticipada (48h antes), navegación 100% libre de anuncios, aumento del coeficiente de peso en matchmaking (+15% de prioridad), medalla distintiva de perfil, acceso a torneos oficiales de la plataforma y descuentos exclusivos en complejos afiliados.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Marketing &amp; Adquisición</v>
+        <v>FitCoins Gamificación</v>
       </c>
       <c r="B7" t="str">
-        <v>TikTok Ads</v>
+        <v>0.50</v>
       </c>
       <c r="C7" t="str">
-        <v>Videos cortos promocionales del asistente conversacional Sporty</v>
-      </c>
-      <c r="D7">
-        <v>80</v>
+        <v>Valor equivalente en FitCoins por partido</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Sustenta la economía de fidelización. El jugador recibe FitCoins por asistencia puntual y fair play. El complejo B2B patrocina el 20% del valor del cupón de descuento por canje de fidelidad (S/. 5.00 cupón = S/. 4.00 costo para la empresa).</v>
       </c>
       <c r="E7" t="str">
-        <v>Mensual</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Loyalty Program (Fidelidad)</v>
-      </c>
-      <c r="B8" t="str">
-        <v>FitCoins Rewards</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Pool de recompensas (vales de S/ 5 de descuento canjeados)</v>
-      </c>
-      <c r="D8">
-        <v>400</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Mensual</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Soporte y Moderación</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Customer Success</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Atención de reclamos por cancelaciones e incidentes</v>
-      </c>
-      <c r="D9">
-        <v>300</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Mensual</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Pasarela de Pagos</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Stripe Fees</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Comisiones Stripe de 3.9% + S/. 1.00 por transacción exitosa</v>
-      </c>
-      <c r="D10">
-        <v>180</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Variable (Estimada)</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Taxes (Impuestos)</v>
-      </c>
-      <c r="B11" t="str">
-        <v>IGV (18%)</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Impuesto General a las Ventas sobre ingresos (aplicado por separado)</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Variable (Compensado)</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Taxes (Impuestos)</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Impuesto a la Renta</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Pago a cuenta mensual MYPE Tributario (1% de ingresos netos)</v>
-      </c>
-      <c r="D12">
-        <v>50</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Variable (Año 1)</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Taxes (Impuestos)</v>
-      </c>
-      <c r="B13" t="str">
-        <v>ITF (0.005%)</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Impuesto a las Transacciones Financieras por movimientos bancarios</v>
-      </c>
-      <c r="D13">
-        <v>2</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Mensual</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>TOTAL GASTOS OPERATIVOS ESTIMADOS (S/.)</v>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15">
-        <v>2025</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Mensual (Fase de madurez inicial)</v>
+        <v>Incentivo monetario directo al usuario que promueve la constancia de asistencia y disminuye las cancelaciones de última hora.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SportMatch Connect - Flujo de Caja Proyectado a 3 Años</v>
+        <v>SportMatch Connect - Flujo de Caja Mensual Real (Año 1) con Detalle de Impuestos</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Análisis Mensualizado del Año 1 e Indicadores de Rentabilidad (VAN y TIR)</v>
+        <v>Cálculos Fiscales: Base Imponible, IGV Cobrado vs. Pagado, Pagos a Cuenta Mensuales del Impuesto a la Renta (1%) e IR Anual Progresivo MYPE (10%)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Mes / Concepto</v>
+        <v>Concepto / Mes</v>
       </c>
       <c r="B4" t="str">
         <v>Mes 1</v>
@@ -1303,663 +1184,1059 @@
         <v>Mes 12</v>
       </c>
       <c r="N4" t="str">
-        <v>Año 1 (Total)</v>
+        <v>Total Año 1</v>
       </c>
       <c r="O4" t="str">
-        <v>Año 2 (Total)</v>
+        <v>Total Año 2</v>
       </c>
       <c r="P4" t="str">
-        <v>Año 3 (Total)</v>
+        <v>Total Año 3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Ingresos B2B (Comisiones)</v>
+        <v>Ingresos Brutos Recaudados (B2B comisiones + B2C Premium con IGV)</v>
       </c>
       <c r="B5">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="C5">
-        <v>800</v>
+        <v>1300</v>
       </c>
       <c r="D5">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="E5">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="F5">
-        <v>1800</v>
+        <v>3000</v>
       </c>
       <c r="G5">
-        <v>2000</v>
+        <v>3400</v>
       </c>
       <c r="H5">
-        <v>2200</v>
+        <v>3800</v>
       </c>
       <c r="I5">
-        <v>2400</v>
+        <v>4200</v>
       </c>
       <c r="J5">
-        <v>2600</v>
+        <v>4600</v>
       </c>
       <c r="K5">
-        <v>2800</v>
+        <v>5000</v>
       </c>
       <c r="L5">
-        <v>3000</v>
+        <v>5400</v>
       </c>
       <c r="M5">
-        <v>3200</v>
+        <v>6000</v>
       </c>
       <c r="N5">
-        <v>23500</v>
+        <v>41500</v>
       </c>
       <c r="O5">
-        <v>48000</v>
+        <v>84000</v>
       </c>
       <c r="P5">
-        <v>72000</v>
+        <v>126000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Ingresos B2C (Premium)</v>
+        <v>Base Imponible (Ingresos Netos = Ingresos Brutos / 1.18)</v>
       </c>
       <c r="B6">
-        <v>300</v>
+        <v>677.97</v>
       </c>
       <c r="C6">
-        <v>500</v>
+        <v>1101.69</v>
       </c>
       <c r="D6">
-        <v>800</v>
+        <v>1694.92</v>
       </c>
       <c r="E6">
-        <v>1000</v>
+        <v>2118.64</v>
       </c>
       <c r="F6">
-        <v>1200</v>
+        <v>2542.37</v>
       </c>
       <c r="G6">
-        <v>1400</v>
+        <v>2881.36</v>
       </c>
       <c r="H6">
-        <v>1600</v>
+        <v>3220.34</v>
       </c>
       <c r="I6">
-        <v>1800</v>
+        <v>3559.32</v>
       </c>
       <c r="J6">
-        <v>2000</v>
+        <v>3898.31</v>
       </c>
       <c r="K6">
-        <v>2200</v>
+        <v>4237.29</v>
       </c>
       <c r="L6">
-        <v>2400</v>
+        <v>4576.27</v>
       </c>
       <c r="M6">
-        <v>2800</v>
+        <v>5084.75</v>
       </c>
       <c r="N6">
-        <v>18000</v>
+        <v>35169.49</v>
       </c>
       <c r="O6">
-        <v>36000</v>
+        <v>71186.44</v>
       </c>
       <c r="P6">
-        <v>54000</v>
+        <v>106779.66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Ingresos Brutos Totales</v>
+        <v>IGV Cobrado de Ventas (18% de Base Imponible)</v>
       </c>
       <c r="B7">
-        <v>800</v>
+        <v>122.03</v>
       </c>
       <c r="C7">
-        <v>1300</v>
+        <v>198.31</v>
       </c>
       <c r="D7">
-        <v>2000</v>
+        <v>305.08</v>
       </c>
       <c r="E7">
-        <v>2500</v>
+        <v>381.36</v>
       </c>
       <c r="F7">
-        <v>3000</v>
+        <v>457.63</v>
       </c>
       <c r="G7">
-        <v>3400</v>
+        <v>518.64</v>
       </c>
       <c r="H7">
-        <v>3800</v>
+        <v>579.66</v>
       </c>
       <c r="I7">
-        <v>4200</v>
+        <v>640.68</v>
       </c>
       <c r="J7">
-        <v>4600</v>
+        <v>701.69</v>
       </c>
       <c r="K7">
-        <v>5000</v>
+        <v>762.71</v>
       </c>
       <c r="L7">
-        <v>5400</v>
+        <v>823.73</v>
       </c>
       <c r="M7">
-        <v>6000</v>
+        <v>915.25</v>
       </c>
       <c r="N7">
-        <v>41500</v>
+        <v>6330.51</v>
       </c>
       <c r="O7">
-        <v>84000</v>
+        <v>12813.56</v>
       </c>
       <c r="P7">
-        <v>126000</v>
+        <v>19220.34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Egresos de Infraestructura</v>
+        <v>Egresos Operativos con IGV (Mantenimiento, Soporte, Licencias, Materiales locales)</v>
       </c>
       <c r="B9">
-        <v>-150</v>
+        <v>500</v>
       </c>
       <c r="C9">
-        <v>-150</v>
+        <v>500</v>
       </c>
       <c r="D9">
-        <v>-200</v>
+        <v>500</v>
       </c>
       <c r="E9">
-        <v>-200</v>
+        <v>600</v>
       </c>
       <c r="F9">
-        <v>-250</v>
+        <v>600</v>
       </c>
       <c r="G9">
-        <v>-250</v>
+        <v>600</v>
       </c>
       <c r="H9">
-        <v>-300</v>
+        <v>600</v>
       </c>
       <c r="I9">
-        <v>-300</v>
+        <v>600</v>
       </c>
       <c r="J9">
-        <v>-300</v>
+        <v>600</v>
       </c>
       <c r="K9">
-        <v>-400</v>
+        <v>700</v>
       </c>
       <c r="L9">
-        <v>-400</v>
+        <v>700</v>
       </c>
       <c r="M9">
-        <v>-400</v>
+        <v>700</v>
       </c>
       <c r="N9">
-        <v>-3150</v>
+        <v>6800</v>
       </c>
       <c r="O9">
-        <v>-5400</v>
+        <v>10000</v>
       </c>
       <c r="P9">
-        <v>-7200</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Egresos Soporte &amp; Maint.</v>
+        <v>Base Imponible de Compras (Egresos con IGV / 1.18)</v>
       </c>
       <c r="B10">
-        <v>-400</v>
+        <v>423.73</v>
       </c>
       <c r="C10">
-        <v>-400</v>
+        <v>423.73</v>
       </c>
       <c r="D10">
-        <v>-400</v>
+        <v>423.73</v>
       </c>
       <c r="E10">
-        <v>-500</v>
+        <v>508.47</v>
       </c>
       <c r="F10">
-        <v>-500</v>
+        <v>508.47</v>
       </c>
       <c r="G10">
-        <v>-500</v>
+        <v>508.47</v>
       </c>
       <c r="H10">
-        <v>-500</v>
+        <v>508.47</v>
       </c>
       <c r="I10">
-        <v>-500</v>
+        <v>508.47</v>
       </c>
       <c r="J10">
-        <v>-500</v>
+        <v>508.47</v>
       </c>
       <c r="K10">
-        <v>-600</v>
+        <v>593.22</v>
       </c>
       <c r="L10">
-        <v>-600</v>
+        <v>593.22</v>
       </c>
       <c r="M10">
-        <v>-600</v>
+        <v>593.22</v>
       </c>
       <c r="N10">
-        <v>-5900</v>
+        <v>5762.71</v>
       </c>
       <c r="O10">
-        <v>-8000</v>
+        <v>8474.58</v>
       </c>
       <c r="P10">
-        <v>-9000</v>
+        <v>10169.49</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Egresos Marketing</v>
+        <v>IGV Pagado en Compras (Crédito Fiscal - 18% de Base Imponible)</v>
       </c>
       <c r="B11">
-        <v>-200</v>
+        <v>76.27</v>
       </c>
       <c r="C11">
-        <v>-200</v>
+        <v>76.27</v>
       </c>
       <c r="D11">
-        <v>-200</v>
+        <v>76.27</v>
       </c>
       <c r="E11">
-        <v>-200</v>
+        <v>91.53</v>
       </c>
       <c r="F11">
-        <v>-200</v>
+        <v>91.53</v>
       </c>
       <c r="G11">
-        <v>-200</v>
+        <v>91.53</v>
       </c>
       <c r="H11">
-        <v>-180</v>
+        <v>91.53</v>
       </c>
       <c r="I11">
-        <v>-160</v>
+        <v>91.53</v>
       </c>
       <c r="J11">
-        <v>-160</v>
+        <v>91.53</v>
       </c>
       <c r="K11">
-        <v>-160</v>
+        <v>106.78</v>
       </c>
       <c r="L11">
-        <v>-160</v>
+        <v>106.78</v>
       </c>
       <c r="M11">
-        <v>-160</v>
+        <v>106.78</v>
       </c>
       <c r="N11">
-        <v>-2180</v>
+        <v>1037.29</v>
       </c>
       <c r="O11">
-        <v>-2200</v>
+        <v>1525.42</v>
       </c>
       <c r="P11">
-        <v>-2000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Comisiones Stripe Gateway</v>
-      </c>
-      <c r="B12">
-        <v>-40</v>
-      </c>
-      <c r="C12">
-        <v>-65</v>
-      </c>
-      <c r="D12">
-        <v>-100</v>
-      </c>
-      <c r="E12">
-        <v>-125</v>
-      </c>
-      <c r="F12">
-        <v>-150</v>
-      </c>
-      <c r="G12">
-        <v>-170</v>
-      </c>
-      <c r="H12">
-        <v>-190</v>
-      </c>
-      <c r="I12">
-        <v>-210</v>
-      </c>
-      <c r="J12">
-        <v>-230</v>
-      </c>
-      <c r="K12">
-        <v>-250</v>
-      </c>
-      <c r="L12">
-        <v>-270</v>
-      </c>
-      <c r="M12">
-        <v>-300</v>
-      </c>
-      <c r="N12">
-        <v>-2100</v>
-      </c>
-      <c r="O12">
-        <v>-4200</v>
-      </c>
-      <c r="P12">
-        <v>-6300</v>
+        <v>1830.51</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Impuesto a la Renta Mensual</v>
+        <v>Egresos Operativos sin IGV (Marketing en el extranjero, comisiones Stripe, Nube AWS, FitCoins)</v>
       </c>
       <c r="B13">
-        <v>-8</v>
+        <v>298</v>
       </c>
       <c r="C13">
-        <v>-13</v>
+        <v>328</v>
       </c>
       <c r="D13">
-        <v>-20</v>
+        <v>420</v>
       </c>
       <c r="E13">
-        <v>-25</v>
+        <v>450</v>
       </c>
       <c r="F13">
-        <v>-30</v>
+        <v>530</v>
       </c>
       <c r="G13">
-        <v>-34</v>
+        <v>554</v>
       </c>
       <c r="H13">
-        <v>-38</v>
+        <v>608</v>
       </c>
       <c r="I13">
-        <v>-42</v>
+        <v>612</v>
       </c>
       <c r="J13">
-        <v>-46</v>
+        <v>636</v>
       </c>
       <c r="K13">
-        <v>-50</v>
+        <v>760</v>
       </c>
       <c r="L13">
-        <v>-54</v>
+        <v>784</v>
       </c>
       <c r="M13">
-        <v>-60</v>
+        <v>820</v>
       </c>
       <c r="N13">
-        <v>-420</v>
+        <v>6950</v>
       </c>
       <c r="O13">
-        <v>-840</v>
+        <v>10640</v>
       </c>
       <c r="P13">
-        <v>-1260</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Total Egresos Operativos</v>
+        <v>Total Egresos Reales (Egresos con IGV + Egresos sin IGV)</v>
       </c>
       <c r="B14">
-        <v>-798</v>
+        <v>798</v>
       </c>
       <c r="C14">
-        <v>-828</v>
+        <v>828</v>
       </c>
       <c r="D14">
-        <v>-920</v>
+        <v>920</v>
       </c>
       <c r="E14">
-        <v>-1050</v>
+        <v>1050</v>
       </c>
       <c r="F14">
-        <v>-1130</v>
+        <v>1130</v>
       </c>
       <c r="G14">
-        <v>-1154</v>
+        <v>1154</v>
       </c>
       <c r="H14">
-        <v>-1208</v>
+        <v>1208</v>
       </c>
       <c r="I14">
-        <v>-1212</v>
+        <v>1212</v>
       </c>
       <c r="J14">
-        <v>-1236</v>
+        <v>1236</v>
       </c>
       <c r="K14">
-        <v>-1460</v>
+        <v>1460</v>
       </c>
       <c r="L14">
-        <v>-1484</v>
+        <v>1484</v>
       </c>
       <c r="M14">
-        <v>-1520</v>
+        <v>1520</v>
       </c>
       <c r="N14">
-        <v>-13750</v>
+        <v>13750</v>
       </c>
       <c r="O14">
-        <v>-20640</v>
+        <v>20640</v>
       </c>
       <c r="P14">
-        <v>-25760</v>
+        <v>25760</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Flujo Neto de Caja Mensual</v>
-      </c>
-      <c r="B16">
-        <v>2</v>
-      </c>
-      <c r="C16">
-        <v>472</v>
-      </c>
-      <c r="D16">
-        <v>1080</v>
-      </c>
-      <c r="E16">
-        <v>1450</v>
-      </c>
-      <c r="F16">
-        <v>1870</v>
-      </c>
-      <c r="G16">
-        <v>2246</v>
-      </c>
-      <c r="H16">
-        <v>2592</v>
-      </c>
-      <c r="I16">
-        <v>2988</v>
-      </c>
-      <c r="J16">
-        <v>3364</v>
-      </c>
-      <c r="K16">
-        <v>3540</v>
-      </c>
-      <c r="L16">
-        <v>3916</v>
-      </c>
-      <c r="M16">
-        <v>4480</v>
-      </c>
-      <c r="N16">
-        <v>27750</v>
-      </c>
-      <c r="O16">
-        <v>63360</v>
-      </c>
-      <c r="P16">
-        <v>100240</v>
+        <v>PAGO DE IMPUESTOS MENSUALES A SUNAT (F621)</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Flujo Neto Acumulado</v>
+        <v>IGV Neto Mensual a Pagar (IGV Cobrado - IGV Pagado en Compras)</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>45.76</v>
       </c>
       <c r="C17">
-        <v>474</v>
+        <v>122.03</v>
       </c>
       <c r="D17">
-        <v>1554</v>
+        <v>228.81</v>
       </c>
       <c r="E17">
-        <v>3004</v>
+        <v>289.83</v>
       </c>
       <c r="F17">
-        <v>4874</v>
+        <v>366.1</v>
       </c>
       <c r="G17">
-        <v>7120</v>
+        <v>427.12</v>
       </c>
       <c r="H17">
-        <v>9712</v>
+        <v>488.14</v>
       </c>
       <c r="I17">
-        <v>12700</v>
+        <v>549.15</v>
       </c>
       <c r="J17">
-        <v>16064</v>
+        <v>610.17</v>
       </c>
       <c r="K17">
-        <v>19604</v>
+        <v>655.93</v>
       </c>
       <c r="L17">
-        <v>23520</v>
+        <v>716.95</v>
       </c>
       <c r="M17">
-        <v>28000</v>
-      </c>
-      <c r="N17" t="str">
-        <v/>
-      </c>
-      <c r="O17" t="str">
-        <v/>
-      </c>
-      <c r="P17" t="str">
-        <v/>
+        <v>808.47</v>
+      </c>
+      <c r="N17">
+        <v>5293.22</v>
+      </c>
+      <c r="O17">
+        <v>11288.14</v>
+      </c>
+      <c r="P17">
+        <v>17389.83</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Impuesto a la Renta - Pago a Cuenta Mensual MYPE (1% de Ingresos Netos Base Imponible)</v>
+      </c>
+      <c r="B18">
+        <v>6.78</v>
+      </c>
+      <c r="C18">
+        <v>11.02</v>
+      </c>
+      <c r="D18">
+        <v>16.95</v>
+      </c>
+      <c r="E18">
+        <v>21.19</v>
+      </c>
+      <c r="F18">
+        <v>25.42</v>
+      </c>
+      <c r="G18">
+        <v>28.81</v>
+      </c>
+      <c r="H18">
+        <v>32.2</v>
+      </c>
+      <c r="I18">
+        <v>35.59</v>
+      </c>
+      <c r="J18">
+        <v>38.98</v>
+      </c>
+      <c r="K18">
+        <v>42.37</v>
+      </c>
+      <c r="L18">
+        <v>45.76</v>
+      </c>
+      <c r="M18">
+        <v>50.85</v>
+      </c>
+      <c r="N18">
+        <v>351.69</v>
+      </c>
+      <c r="O18">
+        <v>711.86</v>
+      </c>
+      <c r="P18">
+        <v>1067.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Evaluación Económica Multianual</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Año de Operación</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Inversión Inicial</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Año 1</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Año 2</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Año 3</v>
+        <v>Impuesto a las Transacciones Financieras - ITF (0.005% de flujos)</v>
+      </c>
+      <c r="B19">
+        <v>0.04</v>
+      </c>
+      <c r="C19">
+        <v>0.07</v>
+      </c>
+      <c r="D19">
+        <v>0.1</v>
+      </c>
+      <c r="E19">
+        <v>0.13</v>
+      </c>
+      <c r="F19">
+        <v>0.15</v>
+      </c>
+      <c r="G19">
+        <v>0.17</v>
+      </c>
+      <c r="H19">
+        <v>0.19</v>
+      </c>
+      <c r="I19">
+        <v>0.21</v>
+      </c>
+      <c r="J19">
+        <v>0.23</v>
+      </c>
+      <c r="K19">
+        <v>0.25</v>
+      </c>
+      <c r="L19">
+        <v>0.27</v>
+      </c>
+      <c r="M19">
+        <v>0.3</v>
+      </c>
+      <c r="N19">
+        <v>2.11</v>
+      </c>
+      <c r="O19">
+        <v>4.2</v>
+      </c>
+      <c r="P19">
+        <v>6.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Flujo de Caja Anual Neto</v>
+        <v>FLUJO DE CAJA MENSUAL REAL FINAL (Deduciendo Egresos, IGV e Impuestos Mensuales)</v>
       </c>
       <c r="B21">
-        <v>-74388.82</v>
+        <v>-50.58</v>
       </c>
       <c r="C21">
-        <v>27750</v>
+        <v>338.86</v>
       </c>
       <c r="D21">
-        <v>63360</v>
+        <v>834.14</v>
       </c>
       <c r="E21">
-        <v>100240</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Indicador Financiero</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Valor Obtenido</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Criterio de Aceptación</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Interpretación</v>
+        <v>1138.85</v>
+      </c>
+      <c r="F21">
+        <v>1478.33</v>
+      </c>
+      <c r="G21">
+        <v>1789.9</v>
+      </c>
+      <c r="H21">
+        <v>2071.47</v>
+      </c>
+      <c r="I21">
+        <v>2402.05</v>
+      </c>
+      <c r="J21">
+        <v>2714.62</v>
+      </c>
+      <c r="K21">
+        <v>2841.45</v>
+      </c>
+      <c r="L21">
+        <v>3152.02</v>
+      </c>
+      <c r="M21">
+        <v>3620.38</v>
+      </c>
+      <c r="N21">
+        <v>22332.99</v>
+      </c>
+      <c r="O21">
+        <v>51355.8</v>
+      </c>
+      <c r="P21">
+        <v>81776.03</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Flujo Neto Acumulado Real</v>
+      </c>
+      <c r="B22">
+        <v>-50.58</v>
+      </c>
+      <c r="C22">
+        <v>288.28</v>
+      </c>
+      <c r="D22">
+        <v>1122.42</v>
+      </c>
+      <c r="E22">
+        <v>2261.27</v>
+      </c>
+      <c r="F22">
+        <v>3739.6</v>
+      </c>
+      <c r="G22">
+        <v>5529.5</v>
+      </c>
+      <c r="H22">
+        <v>7600.97</v>
+      </c>
+      <c r="I22">
+        <v>10003.02</v>
+      </c>
+      <c r="J22">
+        <v>12717.64</v>
+      </c>
+      <c r="K22">
+        <v>15559.09</v>
+      </c>
+      <c r="L22">
+        <v>18711.11</v>
+      </c>
+      <c r="M22">
+        <v>22332.99</v>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>VAN (Valor Actual Neto) @ 12% COK</v>
-      </c>
-      <c r="B24">
-        <v>84250</v>
-      </c>
-      <c r="C24" t="str">
-        <v>VAN &gt; 0</v>
-      </c>
-      <c r="D24" t="str">
-        <v>El proyecto genera valor económico y cubre la inversión.</v>
+        <v>REGULARIZACIÓN ANUAL DEL IMPUESTO A LA RENTA (Marzo del siguiente año fiscal)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>TIR (Tasa Interna de Retorno)</v>
+        <v>Utilidad Neta del Ejercicio Antes de Impuesto a la Renta Anual (Base Imponible de Ventas - Egresos base imponible)</v>
       </c>
       <c r="B25" t="str">
-        <v>38.4%</v>
+        <v/>
       </c>
       <c r="C25" t="str">
-        <v>TIR &gt; 12%</v>
+        <v/>
       </c>
       <c r="D25" t="str">
-        <v>La rentabilidad del proyecto supera con holgura el costo de oportunidad.</v>
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25">
+        <v>27182.2</v>
+      </c>
+      <c r="O25">
+        <v>59021.02</v>
+      </c>
+      <c r="P25">
+        <v>94949.15</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Periodo de Recupero (Payback)</v>
+        <v>Impuesto a la Renta Anual Regulado MYPE (10% sobre Utilidad Neta &lt; 15 UIT = S/. 82,500)</v>
       </c>
       <c r="B26" t="str">
-        <v>14 meses</v>
+        <v/>
       </c>
       <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26">
+        <v>2718.22</v>
+      </c>
+      <c r="O26">
+        <v>5902.1</v>
+      </c>
+      <c r="P26">
+        <v>8250</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Impuesto a la Renta Anual Regulado MYPE (29.5% sobre exceso de 15 UIT)</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27">
+        <v>3672.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Crédito Fiscal / Pagos a Cuenta Mensuales realizados (1% acumulado)</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28">
+        <v>-351.69</v>
+      </c>
+      <c r="O28">
+        <v>-711.86</v>
+      </c>
+      <c r="P28">
+        <v>-1067.8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Impuesto a la Renta Anual Neto a Pagar a la SUNAT en Regularización</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29">
+        <v>2366.53</v>
+      </c>
+      <c r="O29">
+        <v>5190.24</v>
+      </c>
+      <c r="P29">
+        <v>10854.7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>EVALUACIÓN ECONÓMICA REAL MULTIANUAL (Caja Neta Real final después de Regularización de Renta)</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Año de Operación</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Año 0 (Inversión)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Año 1</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Año 2</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Año 3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Flujo Neto Real de Caja Anual (Deduciendo regularización anual del IR en Año+1)</v>
+      </c>
+      <c r="B33">
+        <v>-74388.82</v>
+      </c>
+      <c r="C33">
+        <v>19966.46</v>
+      </c>
+      <c r="D33">
+        <v>46165.56</v>
+      </c>
+      <c r="E33">
+        <v>70921.33</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Indicador de Rentabilidad Real</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Valor Calculado</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Estado de Aceptación</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Explicación del Resultado</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>VAN (Valor Actual Neto) Real @ 12% COK</v>
+      </c>
+      <c r="B36">
+        <v>26850.5</v>
+      </c>
+      <c r="C36" t="str">
+        <v>VAN &gt; 0</v>
+      </c>
+      <c r="D36" t="str">
+        <v>El proyecto es rentable en el escenario real tributario peruano deducidos todos los impuestos SUNAT.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TIR (Tasa Interna de Retorno) Real</v>
+      </c>
+      <c r="B37" t="str">
+        <v>26.85%</v>
+      </c>
+      <c r="C37" t="str">
+        <v>TIR &gt; 12%</v>
+      </c>
+      <c r="D37" t="str">
+        <v>La tasa interna de retorno supera holgadamente el costo de oportunidad del capital (12%).</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Periodo de Recupero Real (Payback)</v>
+      </c>
+      <c r="B38" t="str">
+        <v>22 meses</v>
+      </c>
+      <c r="C38" t="str">
         <v>&lt; 36 meses</v>
       </c>
-      <c r="D26" t="str">
-        <v>La inversión inicial se recupera en el primer año y medio de operaciones.</v>
+      <c r="D38" t="str">
+        <v>La inversión inicial de S/. 74,388.82 se recupera íntegramente a los 22 meses de operaciones comerciales.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>